<commit_message>
the committed capture set, regenerated over the cleaned register
The documents and the walkthrough captures a full suite rewrites, taken from the
run that gated this branch: 74 passed, 1 skipped, 0 failed, NPM_EXIT=0.

They are not cosmetic churn. full-report.csv now carries the staff sentence on
OCVibe and on 4180 Desert Inn, the coverage note no longer claims Clark County
captured nothing on a run that kept 282 records, the register audits count 345
live projects rather than 430, and What moved reads all 1,766 events its
projects hold rather than 1,753.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QVf7gNifkqoKSQrqU1Fh4h
</commit_message>
<xml_diff>
--- a/dashboard/e2e/shots/documents/full-report.xlsx
+++ b/dashboard/e2e/shots/documents/full-report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="189">
   <si>
     <t>Market intelligence report</t>
   </si>
@@ -58,7 +58,7 @@
     <t>ASSESSMENT</t>
   </si>
   <si>
-    <t>This report covers United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 5 projects and 54 captured records. Of those projects, 5 are described in full, selected by significance. 76 projects whose every record has been dismissed are excluded entirely, because they have no filing to cite. 66 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Anything outside that geography or period is not covered here.</t>
+    <t>This report covers United States &gt; Altamonte Springs, Anaheim, Bonita Springs, Central Florida Tourism Oversight District, Clark County, Kissimmee, Lake Buena Vista, Las Vegas, Miami-Dade County, Nashville, Oakland, Phoenix, San Antonio, South Florida, Walt Disney World for July 2026. It is drawn from 5 projects and 54 captured records. Of those projects, 5 are described in full, selected by significance. 65 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Anything outside that geography or period is not covered here.</t>
   </si>
   <si>
     <t>Headline finds</t>
@@ -100,7 +100,7 @@
     <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3618#item-h84e398be28a0</t>
   </si>
   <si>
-    <t>Disneyland Resort: Determination of good faith compliance with the terms and conditions of the First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period for the Disneyland Resort Project</t>
+    <t>Disneyland Resort: Determination that the property owner has complied in good faith with the terms and conditions of the First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period for the Disneyland Resort Project</t>
   </si>
   <si>
     <t>2026-06-22 | Anaheim</t>
@@ -115,201 +115,186 @@
     <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3511#item-h2d4a3a6c3f2a</t>
   </si>
   <si>
-    <t>CFTOD / Walt Disney World: Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement for underground communication lines</t>
+    <t>CFTOD / Walt Disney World: Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
   </si>
   <si>
     <t>2026-01-23 | Central Florida Tourism Oversight District</t>
   </si>
   <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
+  </si>
+  <si>
+    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
+  </si>
+  <si>
+    <t>2026-01-26 | Anaheim</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
+  </si>
+  <si>
+    <t>Entertainment/Attractions</t>
+  </si>
+  <si>
+    <t>OCVibe</t>
+  </si>
+  <si>
+    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
+  </si>
+  <si>
+    <t>Anaheim | approved</t>
+  </si>
+  <si>
+    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC</t>
+  </si>
+  <si>
+    <t>applicant | No phone or email in the record, and no other name alongside it.</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_41028b05c8bbcaff66a50cc1bfacf27e.pdf&amp;view=1#item-h7c785c290138</t>
+  </si>
+  <si>
+    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_7f2f654f7555addc70231de198fa22d9.pdf&amp;view=1#item-h9f002fc7dbca</t>
+  </si>
+  <si>
+    <t>8 further records name the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach. 2 further names on the filings are staff of the body deciding the matter (Lisandro Orozco; Stacy Tran), named there as the case contact and reachable only at that body's own address. They are held in the record and not listed above as a party to approach.</t>
+  </si>
+  <si>
+    <t>2026-02-06. OCVibe Residential Phase I</t>
+  </si>
+  <si>
+    <t>https://ceqanet.lci.ca.gov/Project/2004121045</t>
+  </si>
+  <si>
+    <t>2026-04-20. Approve Amendment No. 2 to Bond Purchase Agreement between the City of Anaheim, the Public Financing Authority, and JP Morgan amending the scheduled completion date to no later than June 25, 2027 for the parking decks associated with the OCVibe Project; and authorize the Finance Director to execute the amendment</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3606#item-h11f1fc13fc80</t>
+  </si>
+  <si>
+    <t>2026-05-05. OCVibe | The new heart of Orange County</t>
+  </si>
+  <si>
+    <t>https://www.ocvibe.com/news/ocvibe-and-award-winning-art-and-design-studio-futureforms-unveil-plans-for-historic-arts-program-in-southern-california</t>
+  </si>
+  <si>
+    <t>2026-05-11. Approve Cooperative Agreement No. 12-0876 with Caltrans for design services and Cooperative Agreement No. 12-0877 with Caltrans for right-of-way services for SR-57 off-ramps</t>
+  </si>
+  <si>
+    <t>2026-05-17. Southern California gets $4B mega music venue in giant...</t>
+  </si>
+  <si>
+    <t>https://nypost.com/2026/05/18/lifestyle/southern-california-lands-mega-venue-in-new-entertainment-district/</t>
+  </si>
+  <si>
+    <t>2026-05-31. First Phase of $4B OCVibe Takes Shape</t>
+  </si>
+  <si>
+    <t>https://www.ocbj.com/oc-homepage/first-phase-of-4b-ocvibe-takes-shape/</t>
+  </si>
+  <si>
+    <t>2026-06-22. 2525 E Katella Ave, Anaheim, CA 92806 - The Weave...</t>
+  </si>
+  <si>
+    <t>https://www.loopnet.com/Listing/2525-E-Katella-Ave-Anaheim-CA/29241061/</t>
+  </si>
+  <si>
+    <t>2026-07-13. Determination that property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No. 2020-00004 for the 2025-2026 review period for the OCVibe Site Master Plan project</t>
+  </si>
+  <si>
+    <t>Players: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE) (applicant)</t>
+  </si>
+  <si>
+    <t>Disneyland Resort</t>
+  </si>
+  <si>
+    <t>Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
+  </si>
+  <si>
+    <t>Records show 4 filings on the first amended and restated development agreement between 2024-05-08 and 2026-06-22.</t>
+  </si>
+  <si>
+    <t>Party: Walt Disney Parks and Resorts U.S., Inc.</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
+  </si>
+  <si>
+    <t>Party: Disneyland</t>
+  </si>
+  <si>
+    <t>https://ceqanet.lci.ca.gov/Project/2021100402</t>
+  </si>
+  <si>
+    <t>Party: Walt Disney Parks and Resorts US, Inc.</t>
+  </si>
+  <si>
+    <t>2 further records name the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+  </si>
+  <si>
+    <t>2024-05-08. DisneylandForward Project</t>
+  </si>
+  <si>
+    <t>Players: Disneyland (applicant)</t>
+  </si>
+  <si>
+    <t>2025-06-16. Determine compliance in good faith with terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2024-2025 review period</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3425#item-h86fdaecda3ed</t>
+  </si>
+  <si>
+    <t>2025-10-27. Approve Cooperative Agreement for funding, design, and construction of Katella Avenue Widening</t>
+  </si>
+  <si>
+    <t>$10,030,000</t>
+  </si>
+  <si>
+    <t>2026-06-22. Determination that the property owner has complied in good faith with the terms and conditions of the First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period for the Disneyland Resort Project</t>
+  </si>
+  <si>
+    <t>Players: Walt Disney Parks and Resorts US, Inc. (applicant)</t>
+  </si>
+  <si>
+    <t>CFTOD / Walt Disney World</t>
+  </si>
+  <si>
+    <t>Records show 3 filings between 2026-01-01 and 2026-01-23.</t>
+  </si>
+  <si>
+    <t>Central Florida Tourism Oversight District | under construction</t>
+  </si>
+  <si>
+    <t>Party: Walt Disney Parks &amp; Resorts U.S. Inc.</t>
+  </si>
+  <si>
     <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.4-p146</t>
   </si>
   <si>
-    <t>Platinum Triangle / PT Metro: Establish new development timeframes and performance time schedule for Development Agreement No. 2005-00008</t>
-  </si>
-  <si>
-    <t>2026-01-26 | Anaheim</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3560#item-h9f77764dd1e5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Development agreement no. 2005-00008 Addendum no. 4 To platinum triangle expansion project mitigation monitoring plan no. 321 Applicant : PT Metro, LLC and Joey Caucas; 20 Enterprise, Suite #125...</t>
-  </si>
-  <si>
-    <t>Entertainment/Attractions</t>
-  </si>
-  <si>
-    <t>OCVibe</t>
-  </si>
-  <si>
-    <t>Approve Cooperative Agreement No. 12-0876, in substantial form, with Caltrans for design (plans, specifications, and estimates) services for the Northbound SR-57 Off-Ramp to Katella Avenue...</t>
-  </si>
-  <si>
-    <t>Anaheim | approved</t>
-  </si>
-  <si>
-    <t>Records show 4 filings and 4 press reports between 2026-02-06 and 2026-07-13.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC</t>
-  </si>
-  <si>
-    <t>applicant | No phone or email in the record, and no other name alongside it.</t>
-  </si>
-  <si>
-    <t>Party: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE)</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_7f2f654f7555addc70231de198fa22d9.pdf&amp;view=1#item-h9f002fc7dbca</t>
-  </si>
-  <si>
-    <t>Party: Lisandro Orozco</t>
-  </si>
-  <si>
-    <t>contact named in the filing | lorozco@anaheim.net</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_45b322ae69423ed7f4d96ffe8e8de725.pdf&amp;view=1#item-h9fe8d90cfc0b</t>
-  </si>
-  <si>
-    <t>Party: Stacy Tran</t>
-  </si>
-  <si>
-    <t>contact named in the filing | STran@anaheim.net</t>
-  </si>
-  <si>
-    <t>https://www.anaheim.net/DocumentCenter/View/66931/Planning-Commission-Action-Agenda---10202025#item-h6dc7e70418cc</t>
-  </si>
-  <si>
-    <t>8 further records name the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
-  </si>
-  <si>
-    <t>2026-02-06. OCVibe Residential Phase I</t>
-  </si>
-  <si>
-    <t>https://ceqanet.lci.ca.gov/Project/2004121045</t>
-  </si>
-  <si>
-    <t>2026-04-20. Approve Amendment No. 2 to Bond Purchase Agreement between the City of Anaheim, the Public Financing Authority, and JP Morgan amending the scheduled completion date to no later than June 25, 2027 for the parking decks associated with the OCVibe Project; and authorize the Finance Director to execute the amendment</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3606#item-h11f1fc13fc80</t>
-  </si>
-  <si>
-    <t>2026-05-05. OCVibe | The new heart of Orange County</t>
-  </si>
-  <si>
-    <t>https://www.ocvibe.com/news/ocvibe-and-award-winning-art-and-design-studio-futureforms-unveil-plans-for-historic-arts-program-in-southern-california</t>
-  </si>
-  <si>
-    <t>2026-05-11. Approve Cooperative Agreement No. 12-0876 with Caltrans for design services and Cooperative Agreement No. 12-0877 with Caltrans for right-of-way services for SR-57 off-ramps</t>
-  </si>
-  <si>
-    <t>2026-05-17. Southern California gets $4B mega music venue in giant...</t>
-  </si>
-  <si>
-    <t>https://nypost.com/2026/05/18/lifestyle/southern-california-lands-mega-venue-in-new-entertainment-district/</t>
-  </si>
-  <si>
-    <t>2026-05-31. First Phase of $4B OCVibe Takes Shape</t>
-  </si>
-  <si>
-    <t>https://www.ocbj.com/oc-homepage/first-phase-of-4b-ocvibe-takes-shape/</t>
-  </si>
-  <si>
-    <t>2026-06-22. 2525 E Katella Ave, Anaheim, CA 92806 - The Weave...</t>
-  </si>
-  <si>
-    <t>https://www.loopnet.com/Listing/2525-E-Katella-Ave-Anaheim-CA/29241061/</t>
-  </si>
-  <si>
-    <t>2026-07-13. Determination that property owner has complied in good faith with the terms and conditions of Amended and Restated Development Agreement No. 2020-00004 for the 2025-2026 review period for the OCVibe Site Master Plan project</t>
-  </si>
-  <si>
-    <t>Players: Anaheim Real Estate Partners, LLC, TS Anaheim, LLC and FCD, LLC (OCVIBE) (applicant)</t>
-  </si>
-  <si>
-    <t>Disneyland Resort</t>
-  </si>
-  <si>
-    <t>Approve the Cooperative Agreement with Walt Disney Parks and Resorts U.S., INC., in the amount estimated at $10,030,000, for funding, design...</t>
-  </si>
-  <si>
-    <t>Records show 4 filings on the first amended and restated development agreement between 2024-05-08 and 2026-06-22.</t>
-  </si>
-  <si>
-    <t>Party: Walt Disney Parks and Resorts U.S., Inc.</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3636#item-h5cf18daa4ec3</t>
-  </si>
-  <si>
-    <t>Party: Disneyland</t>
-  </si>
-  <si>
-    <t>https://ceqanet.lci.ca.gov/Project/2021100402</t>
-  </si>
-  <si>
-    <t>Party: Walt Disney Parks and Resorts US, Inc.</t>
-  </si>
-  <si>
-    <t>One further record names the body that brought this matter forward (City of Anaheim). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
-  </si>
-  <si>
-    <t>2024-05-08. DisneylandForward Project</t>
-  </si>
-  <si>
-    <t>Players: Disneyland (applicant)</t>
-  </si>
-  <si>
-    <t>2025-06-16. Determine compliance in good faith with terms and conditions of First Amended and Restated Development Agreement No. 96-01 for the 2024-2025 review period</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3425#item-h86fdaecda3ed</t>
-  </si>
-  <si>
-    <t>2025-10-27. Approve Cooperative Agreement for funding, design, and construction of Katella Avenue Widening</t>
-  </si>
-  <si>
-    <t>$10,030,000</t>
-  </si>
-  <si>
-    <t>2026-06-22. Determination of good faith compliance with the terms and conditions of the First Amended and Restated Development Agreement No. 96-01 for the 2025-2026 review period for the Disneyland Resort Project</t>
-  </si>
-  <si>
-    <t>Players: Walt Disney Parks and Resorts US, Inc. (applicant)</t>
-  </si>
-  <si>
-    <t>CFTOD / Walt Disney World</t>
-  </si>
-  <si>
-    <t>Records show 3 filings between 2026-01-01 and 2026-01-23.</t>
-  </si>
-  <si>
-    <t>Central Florida Tourism Oversight District | under construction</t>
-  </si>
-  <si>
-    <t>Party: Walt Disney Parks &amp; Resorts U.S. Inc.</t>
-  </si>
-  <si>
-    <t>4 further records name the body that brought this matter forward (Craig Sandt, Director of Construction Management; Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works; Katherine Luetzow, Director, Planning &amp; Engineering). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
-  </si>
-  <si>
-    <t>2026-01-01. CFTOD 2045 Comprehensive Plan - theme park provisions (p.38)</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/2045-CFTOD-Comprehensive-Plan.pdf#plan-p38</t>
+    <t>4 further records name the body that brought this matter forward (Katherine Luetzow, Director, Planning &amp; Engineering Department: Public Works; Craig Sandt, Director of Construction Management). That is who moved it in government rather than who is behind it, so it is not listed above as a party to approach.</t>
+  </si>
+  <si>
+    <t>2026-01-01. CFTOD 2045 Comprehensive Plan - theme park provisions (p.48)</t>
+  </si>
+  <si>
+    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/2045-CFTOD-Comprehensive-Plan.pdf#plan-p48</t>
+  </si>
+  <si>
+    <t>2026-01-23. Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
   </si>
   <si>
     <t>2026-01-23. Approve the District Administrator to execute a Non-exclusive temporary easement with permanent easement for underground communication lines</t>
   </si>
   <si>
-    <t>2026-01-23. Approve the First Amendment to Roadway Expansion Land Dedication and Reimbursement Agreement and authorize the District Administrator or her designee to execute same</t>
-  </si>
-  <si>
-    <t>https://www.oversightdistrict.org/wp-content/uploads/2026/01/1-23-2026-BOS-Agenda-Packet-FINALcs.pdf#item-6.2-p12</t>
-  </si>
-  <si>
     <t>Mixed-Use/Real Estate</t>
   </si>
   <si>
@@ -328,63 +313,57 @@
     <t>applicant | LLC and Joey Caucas | No phone or email in the record.</t>
   </si>
   <si>
-    <t>Party: Christine Nguyen</t>
-  </si>
-  <si>
-    <t>contact named in the filing | CNguyen2@anaheim.net | Also presenter on 2 other projects in our register: 2 in Anaheim.</t>
+    <t>Party: Joey Caucas</t>
+  </si>
+  <si>
+    <t>contact named in the filing | No phone or email in the record, and no other name alongside it.</t>
+  </si>
+  <si>
+    <t>One further name on the filings is staff of the body deciding the matter (Christine Nguyen), named there as the case contact and reachable only at that body's own address. It is held in the record and not listed above as a party to approach.</t>
+  </si>
+  <si>
+    <t>2025-01-13. Adoption of Ordinance No. 6601 amending multiple chapters of Title 18 (Zoning) of the Anaheim Municipal Code and adjustments to multiple specific plans</t>
+  </si>
+  <si>
+    <t>ORDINANCE No. 6601</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3305#item-h9b4b4aa880b3</t>
+  </si>
+  <si>
+    <t>2025-03-23. City-initiated General Plan Amendments to update the General Plan Land Use and Circulation Elements, adopt a new Environmental Justice Element; amendments to Title 18 (Zoning) of the Anaheim Municipal Code; Zoning Reclassification amending the Zoning Map...</t>
+  </si>
+  <si>
+    <t>DEVELOPMENT APPLICATION No. 2021-00223</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_e5a905658061a35b9fb393c9f24d881a.pdf&amp;view=1#item-h0ec28bc385d7</t>
+  </si>
+  <si>
+    <t>2025-04-21. Adopt 2021-2029 Housing Element; update General Plan Land Use, Circulation, and Environmental Justice Elements; amend Title 18 (Zoning) of Anaheim Municipal Code; reclassify zoning; amend Platinum Triangle Master Land Use Plan; adjust Anaheim Canyon Specific Plan No. 2015-1 and Beach Boulevard Specific Plan No...</t>
+  </si>
+  <si>
+    <t>DEVELOPMENT APPLICATION No. 2021-00002</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3384#item-h5b6c84ab98c9</t>
+  </si>
+  <si>
+    <t>2025-05-12. (Adoption) An ordinance of the city of anaheim; amending Chapters 18.06 (Multiple-Family Residential Zones), 18.10 (Industrial Zone), 18.14 (Public and Special-Purpose Zones), 1...</t>
+  </si>
+  <si>
+    <t>ORDINANCE No. 6609</t>
+  </si>
+  <si>
+    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3398#item-h4c01cf1c0349</t>
+  </si>
+  <si>
+    <t>2025-08-10. General Plan Amendment to update the General Plan Land Use Element Table LU-2 (Residential Land Use Designations); amendments to Title 18 (Zoning) of the Anaheim Municipal Code modifying Chapters 18.06 (Multiple-Family Residential Zones), 18.12 (Mixed-Use Zone), and 18.52 (Housing Incentives)</t>
   </si>
   <si>
     <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_2bfcbb0f5f83e7b944ef537de2b1fd4a.pdf&amp;view=1#item-ha13a91a5c59d</t>
   </si>
   <si>
-    <t>Party: Joey Caucas</t>
-  </si>
-  <si>
-    <t>contact named in the filing | No phone or email in the record, and no other name alongside it.</t>
-  </si>
-  <si>
-    <t>2025-01-13. Adoption of Ordinance No. 6601 amending multiple chapters of Title 18 (Zoning) of the Anaheim Municipal Code and adjustments to multiple specific plans</t>
-  </si>
-  <si>
-    <t>ORDINANCE No. 6601</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3305#item-h9b4b4aa880b3</t>
-  </si>
-  <si>
-    <t>2025-03-23. City-initiated General Plan Amendments to update the General Plan Land Use and Circulation Elements, and adopt a new Environmental Justice Element; amendments to Title 18 (Zoning) of the Anaheim Municipal Code; Zoning Reclassification amending the Zoning Map...</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT APPLICATION No. 2021-00223</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/DocumentViewer.php?file=anaheim_e5a905658061a35b9fb393c9f24d881a.pdf&amp;view=1#item-h0ec28bc385d7</t>
-  </si>
-  <si>
-    <t>2025-04-21. Adopt 2021-2029 Housing Element; update General Plan Land Use, Circulation, and Environmental Justice Elements; amend Title 18 (Zoning) of Anaheim Municipal Code; reclassify zoning; amend Platinum Triangle Master Land Use Plan; adjust Anaheim Canyon Specific Plan No. 2015-1 and Beach Boulevard Specific Plan No...</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT APPLICATION No. 2021-00002</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3384#item-h5b6c84ab98c9</t>
-  </si>
-  <si>
-    <t>2025-05-12. (Adoption) An ordinance of the city of anaheim; amending Chapters 18.06 (Multiple-Family Residential Zones), 18.10 (Industrial Zone), 18.14 (Public and Special-Purpose Zones), 1...</t>
-  </si>
-  <si>
-    <t>ORDINANCE No. 6609</t>
-  </si>
-  <si>
-    <t>https://anaheim.granicus.com/AgendaViewer.php?view_id=2&amp;clip_id=3398#item-h4c01cf1c0349</t>
-  </si>
-  <si>
-    <t>2025-08-10. General Plan Amendment to update the General Plan Land Use Element Table LU-2 (Residential Land Use Designations); amendments to Title 18 (Zoning) of the Anaheim Municipal Code modifying Chapters 18.06 (Multiple-Family Residential Zones), 18.12 (Mixed-Use Zone), and 18.52 (Housing Incentives)</t>
-  </si>
-  <si>
-    <t>DEVELOPMENT APPLICATION No. 2021-00223 | Contact: Christine Nguyen. CNguyen2@anaheim.net.</t>
-  </si>
-  <si>
     <t>2025-08-11. Levying Special Taxes within City of Anaheim Community Facilities District No. 06-2 (Stadium Lofts) and Community Facilities District No. 08-1 (Platinum Triangle)</t>
   </si>
   <si>
@@ -436,6 +415,12 @@
     <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=109036</t>
   </si>
   <si>
+    <t>Party: Uncommons Living BLDG 1, LLC</t>
+  </si>
+  <si>
+    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=110657</t>
+  </si>
+  <si>
     <t>Party: 305 Ccd, LLC</t>
   </si>
   <si>
@@ -478,12 +463,6 @@
     <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=107709</t>
   </si>
   <si>
-    <t>Party: Uncommons Living BLDG 1, LLC</t>
-  </si>
-  <si>
-    <t>https://clark.legistar.com/gateway.aspx?M=l&amp;ID=108370</t>
-  </si>
-  <si>
     <t>Party: Nancy Amundsen</t>
   </si>
   <si>
@@ -493,7 +472,7 @@
     <t>Party: Lebene Aidam-ohene</t>
   </si>
   <si>
-    <t>representative | Brown Brown &amp; Premsrirut | 520 S. Fourth Street #200, Las Vegas, NV 89101 | No phone or email in the record.</t>
+    <t>representative | Brown, Brown, &amp; Premsrirut | 520 S. Fourth Street #200, Las Vegas, NV 89101 | No phone or email in the record.</t>
   </si>
   <si>
     <t>Party: Eli Applebaum</t>
@@ -505,7 +484,13 @@
     <t>https://traveltomorrow.com/new-heart-shaped-hotel-approved-for-las-vegas-strip-sparks-debate-over-tacky-design/</t>
   </si>
   <si>
-    <t>2026-05-26. Use permits to expand gaming enterprise district, construct resort hotel, and construct recreational facility; waiver of development standards for non-standard improvements in right-of-way; design review for proposed resort hotel and recreational facility</t>
+    <t>2026-05-26. Tentative map approval for 1 commercial lot on 11.95 acres in a CR (Commercial Resort) Zone within the Airport Environs (AE-60) Overlay</t>
+  </si>
+  <si>
+    <t>TM-26-500056</t>
+  </si>
+  <si>
+    <t>2026-05-26. Use permits to expand gaming enterprise district, develop resort hotel, and recreational facility; waiver of development standards for non-standard improvements in right-of-way; design review for resort hotel and recreational facility</t>
   </si>
   <si>
     <t>UC-26-0219</t>
@@ -514,13 +499,7 @@
     <t>https://www.clarkcountynv.gov/adobe/assets/urn:aaid:aem:bcdf1925-6c37-4308-b6f6-c718c78c9183/original/as/Paradise-Minutes-052626.pdf#item-uc-26-0219</t>
   </si>
   <si>
-    <t>2026-05-26. Tentative map</t>
-  </si>
-  <si>
-    <t>TM-26-500056 | 11.95 acres</t>
-  </si>
-  <si>
-    <t>2026-07-21. Holdover tentative map approval</t>
+    <t>2026-07-21. Holdover tentative map</t>
   </si>
   <si>
     <t>TM-26-500056 | 11.95 acres | Contact: Nancy Amundsen. No phone or email in the record.</t>
@@ -583,7 +562,7 @@
     <t>Dormant projects are excluded from this report. None in this geography is dormant.</t>
   </si>
   <si>
-    <t>66 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Confirming them on the register and regenerating is what puts them in this document.</t>
+    <t>65 projects this scope proposes are held out of this document because they have not been confirmed as part of Simtec Attractions' coverage. A scope is a proposal: it finds projects that look like a match, and each one is confirmed by hand on the register before it may be printed. Those projects are on the register, unconfirmed, and are not a statement that they do not belong here. Confirming them on the register and regenerating is what puts them in this document.</t>
   </si>
   <si>
     <t>This document describes the 15 most significant projects in scope. Every project in scope is described.</t>
@@ -596,9 +575,6 @@
   </si>
   <si>
     <t>12 records counted on the cover are the same filing captured more than once - a bilingual minute, or a document captured page by page - and are shown once above.</t>
-  </si>
-  <si>
-    <t>76 projects in this geography hold no live record and are excluded: every record attached to them has been dismissed on review, so there is nothing to cite.</t>
   </si>
   <si>
     <t>Records are captured from published sources. A matter that has not been published, or that is published somewhere we do not yet capture, will not appear.</t>
@@ -982,7 +958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1299,7 +1275,7 @@
         <v>47</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1313,13 +1289,13 @@
         <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
         <v>47</v>
       </c>
       <c r="F22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1330,16 +1306,16 @@
         <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E23" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F23" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1353,13 +1329,13 @@
         <v>21</v>
       </c>
       <c r="D24" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
         <v>53</v>
-      </c>
-      <c r="E24" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1370,16 +1346,16 @@
         <v>42</v>
       </c>
       <c r="C25" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="F25" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1390,16 +1366,16 @@
         <v>42</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
         <v>57</v>
-      </c>
-      <c r="E26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1413,13 +1389,13 @@
         <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E27" t="s">
         <v>13</v>
       </c>
       <c r="F27" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1433,13 +1409,13 @@
         <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E28" t="s">
         <v>13</v>
       </c>
       <c r="F28" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1450,16 +1426,16 @@
         <v>42</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
       </c>
       <c r="F29" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1473,13 +1449,13 @@
         <v>17</v>
       </c>
       <c r="D30" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
         <v>64</v>
-      </c>
-      <c r="E30" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1490,16 +1466,16 @@
         <v>42</v>
       </c>
       <c r="C31" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D31" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" t="s">
         <v>66</v>
       </c>
-      <c r="E31" t="s">
-        <v>13</v>
-      </c>
       <c r="F31" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1507,19 +1483,19 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D32" t="s">
         <v>68</v>
       </c>
       <c r="E32" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F32" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1527,19 +1503,19 @@
         <v>41</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="F33" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1547,19 +1523,19 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C34" t="s">
         <v>21</v>
       </c>
       <c r="D34" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E34" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F34" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -1567,19 +1543,19 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" t="s">
         <v>72</v>
       </c>
-      <c r="C35" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" t="s">
-        <v>74</v>
-      </c>
       <c r="E35" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F35" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -1587,19 +1563,19 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C36" t="s">
         <v>21</v>
       </c>
       <c r="D36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E36" t="s">
         <v>47</v>
       </c>
       <c r="F36" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1607,19 +1583,19 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E37" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F37" t="s">
-        <v>78</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -1627,19 +1603,19 @@
         <v>41</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C38" t="s">
         <v>21</v>
       </c>
       <c r="D38" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E38" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="F38" t="s">
-        <v>31</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1647,19 +1623,19 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C39" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D39" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E39" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="F39" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1667,19 +1643,19 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C40" t="s">
         <v>21</v>
       </c>
       <c r="D40" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" t="s">
         <v>81</v>
       </c>
-      <c r="E40" t="s">
-        <v>82</v>
-      </c>
       <c r="F40" t="s">
-        <v>78</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1687,19 +1663,19 @@
         <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C41" t="s">
         <v>21</v>
       </c>
       <c r="D41" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41" t="s">
         <v>83</v>
       </c>
-      <c r="E41" t="s">
-        <v>13</v>
-      </c>
       <c r="F41" t="s">
-        <v>84</v>
+        <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1707,10 +1683,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C42" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D42" t="s">
         <v>85</v>
@@ -1719,7 +1695,7 @@
         <v>86</v>
       </c>
       <c r="F42" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1727,7 +1703,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C43" t="s">
         <v>21</v>
@@ -1736,10 +1712,10 @@
         <v>87</v>
       </c>
       <c r="E43" t="s">
+        <v>47</v>
+      </c>
+      <c r="F43" t="s">
         <v>88</v>
-      </c>
-      <c r="F43" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1747,16 +1723,16 @@
         <v>41</v>
       </c>
       <c r="B44" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
         <v>89</v>
       </c>
-      <c r="C44" t="s">
-        <v>13</v>
-      </c>
-      <c r="D44" t="s">
-        <v>90</v>
-      </c>
       <c r="E44" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="F44" t="s">
         <v>13</v>
@@ -1767,19 +1743,19 @@
         <v>41</v>
       </c>
       <c r="B45" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C45" t="s">
         <v>21</v>
       </c>
       <c r="D45" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E45" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="F45" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1787,19 +1763,19 @@
         <v>41</v>
       </c>
       <c r="B46" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C46" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E46" t="s">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="F46" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -1807,27 +1783,27 @@
         <v>41</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C47" t="s">
         <v>21</v>
       </c>
       <c r="D47" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E47" t="s">
         <v>13</v>
       </c>
       <c r="F47" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="B48" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C48" t="s">
         <v>21</v>
@@ -1836,47 +1812,47 @@
         <v>96</v>
       </c>
       <c r="E48" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F48" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C49" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D49" t="s">
         <v>97</v>
       </c>
       <c r="E49" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="F49" t="s">
-        <v>98</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" t="s">
+        <v>98</v>
+      </c>
+      <c r="E50" t="s">
         <v>99</v>
-      </c>
-      <c r="B50" t="s">
-        <v>100</v>
-      </c>
-      <c r="C50" t="s">
-        <v>21</v>
-      </c>
-      <c r="D50" t="s">
-        <v>101</v>
-      </c>
-      <c r="E50" t="s">
-        <v>44</v>
       </c>
       <c r="F50" t="s">
         <v>39</v>
@@ -1884,210 +1860,210 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
+        <v>95</v>
+      </c>
+      <c r="C51" t="s">
+        <v>21</v>
+      </c>
+      <c r="D51" t="s">
         <v>100</v>
       </c>
-      <c r="C51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" t="s">
-        <v>102</v>
-      </c>
       <c r="E51" t="s">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="F51" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C52" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E52" t="s">
-        <v>104</v>
+        <v>44</v>
       </c>
       <c r="F52" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C53" t="s">
         <v>21</v>
       </c>
       <c r="D53" t="s">
+        <v>103</v>
+      </c>
+      <c r="E53" t="s">
+        <v>104</v>
+      </c>
+      <c r="F53" t="s">
         <v>105</v>
-      </c>
-      <c r="E53" t="s">
-        <v>106</v>
-      </c>
-      <c r="F53" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B54" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C54" t="s">
         <v>21</v>
       </c>
       <c r="D54" t="s">
+        <v>106</v>
+      </c>
+      <c r="E54" t="s">
+        <v>107</v>
+      </c>
+      <c r="F54" t="s">
         <v>108</v>
-      </c>
-      <c r="E54" t="s">
-        <v>109</v>
-      </c>
-      <c r="F54" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B55" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C55" t="s">
         <v>21</v>
       </c>
       <c r="D55" t="s">
+        <v>109</v>
+      </c>
+      <c r="E55" t="s">
         <v>110</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
         <v>111</v>
-      </c>
-      <c r="F55" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C56" t="s">
         <v>21</v>
       </c>
       <c r="D56" t="s">
+        <v>112</v>
+      </c>
+      <c r="E56" t="s">
         <v>113</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
         <v>114</v>
-      </c>
-      <c r="F56" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B57" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C57" t="s">
         <v>21</v>
       </c>
       <c r="D57" t="s">
+        <v>115</v>
+      </c>
+      <c r="E57" t="s">
+        <v>107</v>
+      </c>
+      <c r="F57" t="s">
         <v>116</v>
-      </c>
-      <c r="E57" t="s">
-        <v>117</v>
-      </c>
-      <c r="F57" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C58" t="s">
         <v>21</v>
       </c>
       <c r="D58" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E58" t="s">
-        <v>120</v>
+        <v>13</v>
       </c>
       <c r="F58" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C59" t="s">
         <v>21</v>
       </c>
       <c r="D59" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E59" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F59" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B60" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C60" t="s">
         <v>21</v>
       </c>
       <c r="D60" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E60" t="s">
-        <v>13</v>
+        <v>123</v>
       </c>
       <c r="F60" t="s">
-        <v>125</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="B61" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C61" t="s">
         <v>21</v>
@@ -2099,532 +2075,532 @@
         <v>127</v>
       </c>
       <c r="F61" t="s">
-        <v>128</v>
+        <v>23</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="B62" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C62" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E62" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F62" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B63" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C63" t="s">
         <v>21</v>
       </c>
       <c r="D63" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E63" t="s">
-        <v>134</v>
+        <v>47</v>
       </c>
       <c r="F63" t="s">
-        <v>23</v>
+        <v>130</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>124</v>
+      </c>
+      <c r="B64" t="s">
+        <v>125</v>
+      </c>
+      <c r="C64" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" t="s">
         <v>131</v>
       </c>
-      <c r="B64" t="s">
+      <c r="E64" t="s">
         <v>132</v>
       </c>
-      <c r="C64" t="s">
-        <v>13</v>
-      </c>
-      <c r="D64" t="s">
-        <v>135</v>
-      </c>
-      <c r="E64" t="s">
-        <v>134</v>
-      </c>
       <c r="F64" t="s">
-        <v>13</v>
+        <v>133</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B65" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C65" t="s">
         <v>21</v>
       </c>
       <c r="D65" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E65" t="s">
         <v>47</v>
       </c>
       <c r="F65" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C66" t="s">
         <v>21</v>
       </c>
       <c r="D66" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E66" t="s">
-        <v>139</v>
+        <v>47</v>
       </c>
       <c r="F66" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B67" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C67" t="s">
         <v>21</v>
       </c>
       <c r="D67" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E67" t="s">
         <v>47</v>
       </c>
       <c r="F67" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B68" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C68" t="s">
         <v>21</v>
       </c>
       <c r="D68" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E68" t="s">
         <v>47</v>
       </c>
       <c r="F68" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B69" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C69" t="s">
         <v>21</v>
       </c>
       <c r="D69" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E69" t="s">
         <v>47</v>
       </c>
       <c r="F69" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B70" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C70" t="s">
         <v>21</v>
       </c>
       <c r="D70" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E70" t="s">
         <v>47</v>
       </c>
       <c r="F70" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B71" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C71" t="s">
         <v>21</v>
       </c>
       <c r="D71" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E71" t="s">
         <v>47</v>
       </c>
       <c r="F71" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B72" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C72" t="s">
         <v>21</v>
       </c>
       <c r="D72" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="E72" t="s">
         <v>47</v>
       </c>
       <c r="F72" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B73" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C73" t="s">
         <v>21</v>
       </c>
       <c r="D73" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E73" t="s">
-        <v>47</v>
+        <v>151</v>
       </c>
       <c r="F73" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B74" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C74" t="s">
         <v>21</v>
       </c>
       <c r="D74" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E74" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="F74" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B75" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C75" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D75" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E75" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F75" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B76" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C76" t="s">
         <v>21</v>
       </c>
       <c r="D76" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E76" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F76" t="s">
-        <v>150</v>
+        <v>23</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B77" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C77" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D77" t="s">
+        <v>159</v>
+      </c>
+      <c r="E77" t="s">
+        <v>160</v>
+      </c>
+      <c r="F77" t="s">
         <v>161</v>
-      </c>
-      <c r="E77" t="s">
-        <v>162</v>
-      </c>
-      <c r="F77" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B78" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C78" t="s">
         <v>21</v>
       </c>
       <c r="D78" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E78" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F78" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B79" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C79" t="s">
         <v>21</v>
       </c>
       <c r="D79" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E79" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F79" t="s">
-        <v>23</v>
+        <v>166</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B80" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C80" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D80" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E80" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="F80" t="s">
-        <v>137</v>
+        <v>168</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B81" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C81" t="s">
         <v>21</v>
       </c>
       <c r="D81" t="s">
+        <v>169</v>
+      </c>
+      <c r="E81" t="s">
+        <v>170</v>
+      </c>
+      <c r="F81" t="s">
         <v>171</v>
-      </c>
-      <c r="E81" t="s">
-        <v>172</v>
-      </c>
-      <c r="F81" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B82" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C82" t="s">
         <v>17</v>
       </c>
       <c r="D82" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
       </c>
       <c r="F82" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B83" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C83" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D83" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E83" t="s">
-        <v>177</v>
+        <v>13</v>
       </c>
       <c r="F83" t="s">
-        <v>178</v>
+        <v>20</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>131</v>
+        <v>175</v>
       </c>
       <c r="B84" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="C84" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D84" t="s">
-        <v>179</v>
+        <v>24</v>
       </c>
       <c r="E84" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F84" t="s">
-        <v>180</v>
+        <v>26</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>131</v>
+        <v>176</v>
       </c>
       <c r="B85" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="C85" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D85" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E85" t="s">
         <v>13</v>
       </c>
       <c r="F85" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B86" t="s">
         <v>13</v>
       </c>
       <c r="C86" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D86" t="s">
-        <v>24</v>
+        <v>178</v>
       </c>
       <c r="E86" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="F86" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B87" t="s">
         <v>13</v>
       </c>
       <c r="C87" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D87" t="s">
-        <v>18</v>
+        <v>179</v>
       </c>
       <c r="E87" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F87" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B88" t="s">
         <v>13</v>
@@ -2633,7 +2609,7 @@
         <v>14</v>
       </c>
       <c r="D88" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E88" t="s">
         <v>13</v>
@@ -2644,7 +2620,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B89" t="s">
         <v>13</v>
@@ -2653,7 +2629,7 @@
         <v>14</v>
       </c>
       <c r="D89" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E89" t="s">
         <v>13</v>
@@ -2664,7 +2640,7 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B90" t="s">
         <v>13</v>
@@ -2673,7 +2649,7 @@
         <v>14</v>
       </c>
       <c r="D90" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="E90" t="s">
         <v>13</v>
@@ -2684,7 +2660,7 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B91" t="s">
         <v>13</v>
@@ -2693,7 +2669,7 @@
         <v>14</v>
       </c>
       <c r="D91" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E91" t="s">
         <v>13</v>
@@ -2704,7 +2680,7 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B92" t="s">
         <v>13</v>
@@ -2713,7 +2689,7 @@
         <v>14</v>
       </c>
       <c r="D92" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E92" t="s">
         <v>13</v>
@@ -2724,7 +2700,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B93" t="s">
         <v>13</v>
@@ -2733,7 +2709,7 @@
         <v>14</v>
       </c>
       <c r="D93" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E93" t="s">
         <v>13</v>
@@ -2744,7 +2720,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B94" t="s">
         <v>13</v>
@@ -2753,7 +2729,7 @@
         <v>14</v>
       </c>
       <c r="D94" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E94" t="s">
         <v>13</v>
@@ -2764,7 +2740,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B95" t="s">
         <v>13</v>
@@ -2773,7 +2749,7 @@
         <v>14</v>
       </c>
       <c r="D95" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E95" t="s">
         <v>13</v>
@@ -2784,7 +2760,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="B96" t="s">
         <v>13</v>
@@ -2793,92 +2769,12 @@
         <v>14</v>
       </c>
       <c r="D96" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E96" t="s">
         <v>13</v>
       </c>
       <c r="F96" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>183</v>
-      </c>
-      <c r="B97" t="s">
-        <v>13</v>
-      </c>
-      <c r="C97" t="s">
-        <v>14</v>
-      </c>
-      <c r="D97" t="s">
-        <v>193</v>
-      </c>
-      <c r="E97" t="s">
-        <v>13</v>
-      </c>
-      <c r="F97" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>183</v>
-      </c>
-      <c r="B98" t="s">
-        <v>13</v>
-      </c>
-      <c r="C98" t="s">
-        <v>14</v>
-      </c>
-      <c r="D98" t="s">
-        <v>194</v>
-      </c>
-      <c r="E98" t="s">
-        <v>13</v>
-      </c>
-      <c r="F98" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>183</v>
-      </c>
-      <c r="B99" t="s">
-        <v>13</v>
-      </c>
-      <c r="C99" t="s">
-        <v>14</v>
-      </c>
-      <c r="D99" t="s">
-        <v>195</v>
-      </c>
-      <c r="E99" t="s">
-        <v>13</v>
-      </c>
-      <c r="F99" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>183</v>
-      </c>
-      <c r="B100" t="s">
-        <v>13</v>
-      </c>
-      <c r="C100" t="s">
-        <v>14</v>
-      </c>
-      <c r="D100" t="s">
-        <v>196</v>
-      </c>
-      <c r="E100" t="s">
-        <v>13</v>
-      </c>
-      <c r="F100" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>